<commit_message>
Initial commit: Push entire project to GitHub
</commit_message>
<xml_diff>
--- a/docx/需求分析/需求分析矩阵.xlsx
+++ b/docx/需求分析/需求分析矩阵.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\edge下载\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\原神攻略系统\getee-yuanshen\docx\需求分析\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9535F297-12B1-4FB1-AE46-0D09F88F4197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E09D6AA6-C653-41EE-AC3D-734747F9BBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4140" yWindow="2280" windowWidth="17940" windowHeight="13050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="我现在想做一个原神攻略的系统，来放到我的getee上面来作为j" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>